<commit_message>
updated testing method on first slide of excel
</commit_message>
<xml_diff>
--- a/docs/Lab02/Lab02_BBT_TCs_Form.xlsx
+++ b/docs/Lab02/Lab02_BBT_TCs_Form.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42F66CDF-2D0F-4C9E-A568-0C83DADAFFE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE1128C-7222-452A-A5AB-D6205B85212A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="1725" windowWidth="28800" windowHeight="15345" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="1" r:id="rId1"/>
@@ -1069,7 +1069,7 @@
     <t>Stanca Vlad Tudor</t>
   </si>
   <si>
-    <t>updateProduct(String title, String director, int year, List&lt;String&gt; actors, String category, List&lt;String&gt; keywords): void</t>
+    <t>updateProduct(int id, String nume, double pret, String categorie, String tip): void</t>
   </si>
 </sst>
 </file>
@@ -1974,22 +1974,151 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2007,36 +2136,12 @@
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2061,109 +2166,28 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2172,44 +2196,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2608,12 +2608,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="C1" s="81" t="s">
+      <c r="C1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="83"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="105"/>
+      <c r="F1" s="106"/>
       <c r="H1" s="51" t="s">
         <v>1</v>
       </c>
@@ -2621,11 +2621,11 @@
       <c r="J1" s="51"/>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="H2" s="84" t="s">
+      <c r="H2" s="123" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H3" s="2"/>
@@ -2784,21 +2784,21 @@
     </row>
     <row r="24" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="48"/>
-      <c r="B24" s="80" t="s">
+      <c r="B24" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="80"/>
-      <c r="D24" s="80"/>
-      <c r="E24" s="80"/>
-      <c r="F24" s="80"/>
-      <c r="G24" s="80"/>
-      <c r="H24" s="80"/>
-      <c r="I24" s="80"/>
-      <c r="J24" s="80"/>
-      <c r="K24" s="80"/>
-      <c r="L24" s="80"/>
-      <c r="M24" s="80"/>
-      <c r="N24" s="80"/>
+      <c r="C24" s="122"/>
+      <c r="D24" s="122"/>
+      <c r="E24" s="122"/>
+      <c r="F24" s="122"/>
+      <c r="G24" s="122"/>
+      <c r="H24" s="122"/>
+      <c r="I24" s="122"/>
+      <c r="J24" s="122"/>
+      <c r="K24" s="122"/>
+      <c r="L24" s="122"/>
+      <c r="M24" s="122"/>
+      <c r="N24" s="122"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C26" s="50"/>
@@ -2837,39 +2837,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="83"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="106"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="129" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="88"/>
+      <c r="C3" s="130"/>
+      <c r="D3" s="130"/>
+      <c r="E3" s="130"/>
+      <c r="F3" s="130"/>
+      <c r="G3" s="131"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="89" t="s">
+      <c r="B5" s="132" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="89"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="89"/>
-      <c r="G5" s="90" t="s">
+      <c r="C5" s="132"/>
+      <c r="D5" s="132"/>
+      <c r="E5" s="132"/>
+      <c r="G5" s="133" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
-      <c r="K5" s="90"/>
-      <c r="L5" s="90"/>
-      <c r="M5" s="90"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="133"/>
+      <c r="K5" s="133"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="133"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="23" t="s">
@@ -2884,18 +2884,18 @@
       <c r="E6" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="93" t="s">
+      <c r="H6" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="95" t="s">
+      <c r="I6" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="96"/>
-      <c r="K6" s="96"/>
-      <c r="L6" s="96"/>
+      <c r="J6" s="117"/>
+      <c r="K6" s="117"/>
+      <c r="L6" s="117"/>
       <c r="M6" s="23" t="s">
         <v>30</v>
       </c>
@@ -2904,15 +2904,15 @@
       <c r="B7" s="4">
         <v>1</v>
       </c>
-      <c r="C7" s="97" t="s">
+      <c r="C7" s="124" t="s">
         <v>132</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>132</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="G7" s="92"/>
-      <c r="H7" s="94"/>
+      <c r="G7" s="134"/>
+      <c r="H7" s="135"/>
       <c r="I7" s="23" t="s">
         <v>140</v>
       </c>
@@ -2933,7 +2933,7 @@
       <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="97"/>
+      <c r="C8" s="124"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
         <v>133</v>
@@ -2964,7 +2964,7 @@
       <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="85" t="s">
+      <c r="C9" s="128" t="s">
         <v>134</v>
       </c>
       <c r="D9" s="60" t="s">
@@ -2997,7 +2997,7 @@
       <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="85"/>
+      <c r="C10" s="128"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>139</v>
@@ -3028,7 +3028,7 @@
       <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="97" t="s">
+      <c r="C11" s="124" t="s">
         <v>135</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -3061,7 +3061,7 @@
       <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="97"/>
+      <c r="C12" s="124"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
         <v>136</v>
@@ -3092,7 +3092,7 @@
       <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="99" t="s">
+      <c r="C13" s="126" t="s">
         <v>137</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -3113,7 +3113,7 @@
       <c r="B14" s="4">
         <v>8</v>
       </c>
-      <c r="C14" s="100"/>
+      <c r="C14" s="127"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
         <v>138</v>
@@ -3132,7 +3132,7 @@
       <c r="B15" s="4">
         <v>9</v>
       </c>
-      <c r="C15" s="97" t="s">
+      <c r="C15" s="124" t="s">
         <v>49</v>
       </c>
       <c r="D15" s="4"/>
@@ -3151,7 +3151,7 @@
       <c r="B16" s="4">
         <v>10</v>
       </c>
-      <c r="C16" s="97"/>
+      <c r="C16" s="124"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="G16" s="19">
@@ -3168,7 +3168,7 @@
       <c r="B17" s="4">
         <v>11</v>
       </c>
-      <c r="C17" s="97" t="s">
+      <c r="C17" s="124" t="s">
         <v>49</v>
       </c>
       <c r="D17" s="4"/>
@@ -3185,7 +3185,7 @@
       <c r="B18" s="4">
         <v>12</v>
       </c>
-      <c r="C18" s="97"/>
+      <c r="C18" s="124"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="G18" s="19"/>
@@ -3200,7 +3200,7 @@
       <c r="B19" s="4">
         <v>13</v>
       </c>
-      <c r="C19" s="97" t="s">
+      <c r="C19" s="124" t="s">
         <v>49</v>
       </c>
       <c r="D19" s="4"/>
@@ -3217,7 +3217,7 @@
       <c r="B20" s="4">
         <v>14</v>
       </c>
-      <c r="C20" s="97"/>
+      <c r="C20" s="124"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
@@ -3225,8 +3225,8 @@
       <c r="D22" t="s">
         <v>65</v>
       </c>
-      <c r="F22" s="98"/>
-      <c r="G22" s="98"/>
+      <c r="F22" s="125"/>
+      <c r="G22" s="125"/>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.25">
       <c r="M24" s="66"/>
@@ -3236,12 +3236,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="C13:C14"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B3:G3"/>
@@ -3251,6 +3245,12 @@
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="I6:L6"/>
     <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C13:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3281,41 +3281,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="83"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="106"/>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="105" t="s">
+      <c r="B3" s="140" t="s">
         <v>151</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="88"/>
+      <c r="C3" s="130"/>
+      <c r="D3" s="130"/>
+      <c r="E3" s="130"/>
+      <c r="F3" s="130"/>
+      <c r="G3" s="131"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B5" s="106" t="s">
+      <c r="B5" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="106"/>
-      <c r="D5" s="106"/>
+      <c r="C5" s="141"/>
+      <c r="D5" s="141"/>
       <c r="E5" s="3"/>
-      <c r="G5" s="90" t="s">
+      <c r="G5" s="133" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
-      <c r="K5" s="90"/>
-      <c r="L5" s="90"/>
-      <c r="M5" s="90"/>
-      <c r="N5" s="90"/>
-      <c r="O5" s="90"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="133"/>
+      <c r="K5" s="133"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="133"/>
+      <c r="N5" s="133"/>
+      <c r="O5" s="133"/>
     </row>
     <row r="6" spans="2:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
@@ -3328,42 +3328,42 @@
         <v>66</v>
       </c>
       <c r="E6" s="10"/>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="108" t="s">
         <v>69</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="108" t="s">
         <v>70</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="108" t="s">
         <v>71</v>
       </c>
-      <c r="J6" s="93" t="s">
+      <c r="J6" s="114" t="s">
         <v>72</v>
       </c>
-      <c r="K6" s="107" t="s">
+      <c r="K6" s="142" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="108"/>
-      <c r="M6" s="108"/>
-      <c r="N6" s="108"/>
+      <c r="L6" s="143"/>
+      <c r="M6" s="143"/>
+      <c r="N6" s="143"/>
       <c r="O6" s="56" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="99">
+      <c r="B7" s="126">
         <v>1</v>
       </c>
-      <c r="C7" s="102" t="s">
+      <c r="C7" s="137" t="s">
         <v>152</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G7" s="92"/>
-      <c r="H7" s="92"/>
-      <c r="I7" s="92"/>
-      <c r="J7" s="94"/>
+      <c r="G7" s="134"/>
+      <c r="H7" s="134"/>
+      <c r="I7" s="134"/>
+      <c r="J7" s="135"/>
       <c r="K7" s="23" t="s">
         <v>140</v>
       </c>
@@ -3381,8 +3381,8 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="101"/>
-      <c r="C8" s="103"/>
+      <c r="B8" s="136"/>
+      <c r="C8" s="138"/>
       <c r="D8" s="2" t="s">
         <v>154</v>
       </c>
@@ -3413,8 +3413,8 @@
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="101"/>
-      <c r="C9" s="103"/>
+      <c r="B9" s="136"/>
+      <c r="C9" s="138"/>
       <c r="D9" s="2" t="s">
         <v>155</v>
       </c>
@@ -3447,8 +3447,8 @@
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="101"/>
-      <c r="C10" s="103"/>
+      <c r="B10" s="136"/>
+      <c r="C10" s="138"/>
       <c r="D10" s="2" t="s">
         <v>156</v>
       </c>
@@ -3479,8 +3479,8 @@
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="101"/>
-      <c r="C11" s="103"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="138"/>
       <c r="D11" s="2" t="s">
         <v>157</v>
       </c>
@@ -3511,8 +3511,8 @@
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="100"/>
-      <c r="C12" s="104"/>
+      <c r="B12" s="127"/>
+      <c r="C12" s="139"/>
       <c r="D12" s="2" t="s">
         <v>158</v>
       </c>
@@ -3543,10 +3543,10 @@
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="99">
+      <c r="B13" s="126">
         <v>2</v>
       </c>
-      <c r="C13" s="102" t="s">
+      <c r="C13" s="137" t="s">
         <v>134</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -3581,8 +3581,8 @@
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="101"/>
-      <c r="C14" s="103"/>
+      <c r="B14" s="136"/>
+      <c r="C14" s="138"/>
       <c r="D14" s="2" t="s">
         <v>160</v>
       </c>
@@ -3613,8 +3613,8 @@
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="101"/>
-      <c r="C15" s="103"/>
+      <c r="B15" s="136"/>
+      <c r="C15" s="138"/>
       <c r="D15" s="2" t="s">
         <v>161</v>
       </c>
@@ -3645,8 +3645,8 @@
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="101"/>
-      <c r="C16" s="103"/>
+      <c r="B16" s="136"/>
+      <c r="C16" s="138"/>
       <c r="D16" s="2" t="s">
         <v>162</v>
       </c>
@@ -3677,8 +3677,8 @@
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="101"/>
-      <c r="C17" s="103"/>
+      <c r="B17" s="136"/>
+      <c r="C17" s="138"/>
       <c r="D17" s="2" t="s">
         <v>163</v>
       </c>
@@ -3709,8 +3709,8 @@
       </c>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="100"/>
-      <c r="C18" s="104"/>
+      <c r="B18" s="127"/>
+      <c r="C18" s="139"/>
       <c r="D18" s="2" t="s">
         <v>164</v>
       </c>
@@ -3743,10 +3743,10 @@
       </c>
     </row>
     <row r="19" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="99">
+      <c r="B19" s="126">
         <v>3</v>
       </c>
-      <c r="C19" s="102" t="s">
+      <c r="C19" s="137" t="s">
         <v>135</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -3779,8 +3779,8 @@
       </c>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B20" s="101"/>
-      <c r="C20" s="103"/>
+      <c r="B20" s="136"/>
+      <c r="C20" s="138"/>
       <c r="D20" s="2" t="s">
         <v>177</v>
       </c>
@@ -3811,8 +3811,8 @@
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B21" s="101"/>
-      <c r="C21" s="103"/>
+      <c r="B21" s="136"/>
+      <c r="C21" s="138"/>
       <c r="D21" s="2" t="s">
         <v>178</v>
       </c>
@@ -3845,8 +3845,8 @@
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="101"/>
-      <c r="C22" s="103"/>
+      <c r="B22" s="136"/>
+      <c r="C22" s="138"/>
       <c r="D22" s="2" t="s">
         <v>179</v>
       </c>
@@ -3877,8 +3877,8 @@
       </c>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="101"/>
-      <c r="C23" s="103"/>
+      <c r="B23" s="136"/>
+      <c r="C23" s="138"/>
       <c r="D23" s="2" t="s">
         <v>180</v>
       </c>
@@ -3909,8 +3909,8 @@
       </c>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="100"/>
-      <c r="C24" s="104"/>
+      <c r="B24" s="127"/>
+      <c r="C24" s="139"/>
       <c r="D24" s="2" t="s">
         <v>181</v>
       </c>
@@ -3941,10 +3941,10 @@
       </c>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="99">
+      <c r="B25" s="126">
         <v>4</v>
       </c>
-      <c r="C25" s="102" t="s">
+      <c r="C25" s="137" t="s">
         <v>137</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -3979,8 +3979,8 @@
       </c>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="101"/>
-      <c r="C26" s="103"/>
+      <c r="B26" s="136"/>
+      <c r="C26" s="138"/>
       <c r="D26" s="2" t="s">
         <v>183</v>
       </c>
@@ -4011,8 +4011,8 @@
       </c>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B27" s="101"/>
-      <c r="C27" s="103"/>
+      <c r="B27" s="136"/>
+      <c r="C27" s="138"/>
       <c r="D27" s="2" t="s">
         <v>184</v>
       </c>
@@ -4045,8 +4045,8 @@
       </c>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B28" s="101"/>
-      <c r="C28" s="103"/>
+      <c r="B28" s="136"/>
+      <c r="C28" s="138"/>
       <c r="D28" s="2" t="s">
         <v>185</v>
       </c>
@@ -4077,8 +4077,8 @@
       </c>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B29" s="101"/>
-      <c r="C29" s="103"/>
+      <c r="B29" s="136"/>
+      <c r="C29" s="138"/>
       <c r="D29" s="2" t="s">
         <v>186</v>
       </c>
@@ -4109,8 +4109,8 @@
       </c>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B30" s="100"/>
-      <c r="C30" s="104"/>
+      <c r="B30" s="127"/>
+      <c r="C30" s="139"/>
       <c r="D30" s="2" t="s">
         <v>187</v>
       </c>
@@ -4171,12 +4171,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B25:B30"/>
-    <mergeCell ref="C25:C30"/>
-    <mergeCell ref="B19:B24"/>
-    <mergeCell ref="C19:C24"/>
-    <mergeCell ref="B13:B18"/>
-    <mergeCell ref="C13:C18"/>
     <mergeCell ref="B7:B12"/>
     <mergeCell ref="C7:C12"/>
     <mergeCell ref="B1:E1"/>
@@ -4188,6 +4182,12 @@
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:N6"/>
+    <mergeCell ref="B25:B30"/>
+    <mergeCell ref="C25:C30"/>
+    <mergeCell ref="B19:B24"/>
+    <mergeCell ref="C19:C24"/>
+    <mergeCell ref="B13:B18"/>
+    <mergeCell ref="C13:C18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4214,51 +4214,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="83"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="106"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="111" t="s">
+      <c r="B3" s="107" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
-      <c r="M3" s="111"/>
-      <c r="N3" s="111"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="107"/>
+      <c r="L3" s="107"/>
+      <c r="M3" s="107"/>
+      <c r="N3" s="107"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="108" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="113" t="s">
+      <c r="C4" s="110" t="s">
         <v>105</v>
       </c>
-      <c r="D4" s="115" t="s">
+      <c r="D4" s="112" t="s">
         <v>106</v>
       </c>
-      <c r="E4" s="93" t="s">
+      <c r="E4" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="95" t="s">
+      <c r="F4" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="96"/>
-      <c r="H4" s="96"/>
-      <c r="I4" s="96"/>
-      <c r="J4" s="96"/>
-      <c r="K4" s="96"/>
+      <c r="G4" s="117"/>
+      <c r="H4" s="117"/>
+      <c r="I4" s="117"/>
+      <c r="J4" s="117"/>
+      <c r="K4" s="117"/>
       <c r="L4" s="118"/>
       <c r="M4" s="119" t="s">
         <v>30</v>
@@ -4266,10 +4266,10 @@
       <c r="N4" s="119"/>
     </row>
     <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="112"/>
-      <c r="C5" s="114"/>
-      <c r="D5" s="116"/>
-      <c r="E5" s="117"/>
+      <c r="B5" s="109"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="115"/>
       <c r="F5" s="26" t="s">
         <v>140</v>
       </c>
@@ -4296,7 +4296,7 @@
       <c r="B6" s="24">
         <v>1</v>
       </c>
-      <c r="C6" s="109" t="s">
+      <c r="C6" s="102" t="s">
         <v>109</v>
       </c>
       <c r="D6" s="30" t="s">
@@ -4329,7 +4329,7 @@
       <c r="B7" s="12">
         <v>2</v>
       </c>
-      <c r="C7" s="109"/>
+      <c r="C7" s="102"/>
       <c r="D7" s="31" t="s">
         <v>200</v>
       </c>
@@ -4360,7 +4360,7 @@
       <c r="B8" s="24">
         <v>3</v>
       </c>
-      <c r="C8" s="109"/>
+      <c r="C8" s="102"/>
       <c r="D8" s="31" t="s">
         <v>201</v>
       </c>
@@ -4391,7 +4391,7 @@
       <c r="B9" s="24">
         <v>4</v>
       </c>
-      <c r="C9" s="109"/>
+      <c r="C9" s="102"/>
       <c r="D9" s="30" t="s">
         <v>202</v>
       </c>
@@ -4422,7 +4422,7 @@
       <c r="B10" s="12">
         <v>5</v>
       </c>
-      <c r="C10" s="109"/>
+      <c r="C10" s="102"/>
       <c r="D10" s="30" t="s">
         <v>203</v>
       </c>
@@ -4453,7 +4453,7 @@
       <c r="B11" s="24">
         <v>6</v>
       </c>
-      <c r="C11" s="109"/>
+      <c r="C11" s="102"/>
       <c r="D11" s="31" t="s">
         <v>49</v>
       </c>
@@ -4473,8 +4473,8 @@
         <v>50</v>
       </c>
       <c r="J11" s="12"/>
-      <c r="K11" s="131"/>
-      <c r="L11" s="132"/>
+      <c r="K11" s="120"/>
+      <c r="L11" s="121"/>
       <c r="M11" s="12" t="s">
         <v>49</v>
       </c>
@@ -4484,7 +4484,7 @@
       <c r="B12" s="24">
         <v>7</v>
       </c>
-      <c r="C12" s="109"/>
+      <c r="C12" s="102"/>
       <c r="D12" s="31" t="s">
         <v>65</v>
       </c>
@@ -4516,7 +4516,7 @@
       <c r="B13" s="12">
         <v>8</v>
       </c>
-      <c r="C13" s="109"/>
+      <c r="C13" s="102"/>
       <c r="D13" s="31"/>
       <c r="E13" s="12" t="str">
         <f t="shared" ref="E13:E35" si="0">"TC" &amp; (B13 - 6) &amp; "_BVA"</f>
@@ -4546,7 +4546,7 @@
       <c r="B14" s="24">
         <v>9</v>
       </c>
-      <c r="C14" s="109"/>
+      <c r="C14" s="102"/>
       <c r="D14" s="31"/>
       <c r="E14" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4576,7 +4576,7 @@
       <c r="B15" s="12">
         <v>10</v>
       </c>
-      <c r="C15" s="109"/>
+      <c r="C15" s="102"/>
       <c r="D15" s="31"/>
       <c r="E15" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4606,7 +4606,7 @@
       <c r="B16" s="24">
         <v>11</v>
       </c>
-      <c r="C16" s="109"/>
+      <c r="C16" s="102"/>
       <c r="D16" s="31"/>
       <c r="E16" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4636,7 +4636,7 @@
       <c r="B17" s="24">
         <v>12</v>
       </c>
-      <c r="C17" s="109"/>
+      <c r="C17" s="102"/>
       <c r="D17" s="31"/>
       <c r="E17" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4666,7 +4666,7 @@
       <c r="B18" s="12">
         <v>13</v>
       </c>
-      <c r="C18" s="109"/>
+      <c r="C18" s="102"/>
       <c r="D18" s="31"/>
       <c r="E18" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4696,7 +4696,7 @@
       <c r="B19" s="24">
         <v>14</v>
       </c>
-      <c r="C19" s="109"/>
+      <c r="C19" s="102"/>
       <c r="D19" s="31"/>
       <c r="E19" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4726,7 +4726,7 @@
       <c r="B20" s="24">
         <v>15</v>
       </c>
-      <c r="C20" s="109"/>
+      <c r="C20" s="102"/>
       <c r="D20" s="31"/>
       <c r="E20" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4756,7 +4756,7 @@
       <c r="B21" s="12">
         <v>16</v>
       </c>
-      <c r="C21" s="109"/>
+      <c r="C21" s="102"/>
       <c r="D21" s="31"/>
       <c r="E21" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4786,7 +4786,7 @@
       <c r="B22" s="24">
         <v>17</v>
       </c>
-      <c r="C22" s="109"/>
+      <c r="C22" s="102"/>
       <c r="D22" s="31"/>
       <c r="E22" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4816,7 +4816,7 @@
       <c r="B23" s="12">
         <v>18</v>
       </c>
-      <c r="C23" s="109"/>
+      <c r="C23" s="102"/>
       <c r="D23" s="31"/>
       <c r="E23" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4846,7 +4846,7 @@
       <c r="B24" s="24">
         <v>19</v>
       </c>
-      <c r="C24" s="109"/>
+      <c r="C24" s="102"/>
       <c r="D24" s="31"/>
       <c r="E24" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4876,7 +4876,7 @@
       <c r="B25" s="24">
         <v>20</v>
       </c>
-      <c r="C25" s="109"/>
+      <c r="C25" s="102"/>
       <c r="D25" s="31"/>
       <c r="E25" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4906,7 +4906,7 @@
       <c r="B26" s="12">
         <v>21</v>
       </c>
-      <c r="C26" s="109"/>
+      <c r="C26" s="102"/>
       <c r="D26" s="31"/>
       <c r="E26" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4936,7 +4936,7 @@
       <c r="B27" s="24">
         <v>22</v>
       </c>
-      <c r="C27" s="109"/>
+      <c r="C27" s="102"/>
       <c r="D27" s="31"/>
       <c r="E27" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4966,7 +4966,7 @@
       <c r="B28" s="24">
         <v>23</v>
       </c>
-      <c r="C28" s="109"/>
+      <c r="C28" s="102"/>
       <c r="D28" s="31"/>
       <c r="E28" s="12" t="str">
         <f t="shared" si="0"/>
@@ -4996,7 +4996,7 @@
       <c r="B29" s="12">
         <v>24</v>
       </c>
-      <c r="C29" s="109"/>
+      <c r="C29" s="102"/>
       <c r="D29" s="31"/>
       <c r="E29" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5026,7 +5026,7 @@
       <c r="B30" s="24">
         <v>25</v>
       </c>
-      <c r="C30" s="109"/>
+      <c r="C30" s="102"/>
       <c r="D30" s="31"/>
       <c r="E30" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5056,7 +5056,7 @@
       <c r="B31" s="12">
         <v>26</v>
       </c>
-      <c r="C31" s="109"/>
+      <c r="C31" s="102"/>
       <c r="D31" s="31"/>
       <c r="E31" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5086,7 +5086,7 @@
       <c r="B32" s="24">
         <v>27</v>
       </c>
-      <c r="C32" s="109"/>
+      <c r="C32" s="102"/>
       <c r="D32" s="31"/>
       <c r="E32" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5105,8 +5105,8 @@
         <v>81</v>
       </c>
       <c r="J32" s="11"/>
-      <c r="K32" s="129"/>
-      <c r="L32" s="130"/>
+      <c r="K32" s="84"/>
+      <c r="L32" s="85"/>
       <c r="M32" s="57" t="s">
         <v>144</v>
       </c>
@@ -5116,7 +5116,7 @@
       <c r="B33" s="24">
         <v>28</v>
       </c>
-      <c r="C33" s="109"/>
+      <c r="C33" s="102"/>
       <c r="D33" s="31"/>
       <c r="E33" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5135,8 +5135,8 @@
         <v>167</v>
       </c>
       <c r="J33" s="11"/>
-      <c r="K33" s="129"/>
-      <c r="L33" s="130"/>
+      <c r="K33" s="84"/>
+      <c r="L33" s="85"/>
       <c r="M33" s="57" t="s">
         <v>144</v>
       </c>
@@ -5146,7 +5146,7 @@
       <c r="B34" s="12">
         <v>29</v>
       </c>
-      <c r="C34" s="109"/>
+      <c r="C34" s="102"/>
       <c r="D34" s="31"/>
       <c r="E34" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5165,8 +5165,8 @@
         <v>168</v>
       </c>
       <c r="J34" s="11"/>
-      <c r="K34" s="129"/>
-      <c r="L34" s="130"/>
+      <c r="K34" s="84"/>
+      <c r="L34" s="85"/>
       <c r="M34" s="57" t="s">
         <v>144</v>
       </c>
@@ -5176,7 +5176,7 @@
       <c r="B35" s="24">
         <v>30</v>
       </c>
-      <c r="C35" s="110"/>
+      <c r="C35" s="103"/>
       <c r="D35" s="32"/>
       <c r="E35" s="12" t="str">
         <f t="shared" si="0"/>
@@ -5195,8 +5195,8 @@
         <v>169</v>
       </c>
       <c r="J35" s="25"/>
-      <c r="K35" s="135"/>
-      <c r="L35" s="136"/>
+      <c r="K35" s="82"/>
+      <c r="L35" s="83"/>
       <c r="M35" s="53" t="s">
         <v>61</v>
       </c>
@@ -5229,98 +5229,98 @@
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
-      <c r="K37" s="143"/>
-      <c r="L37" s="143"/>
+      <c r="K37" s="92"/>
+      <c r="L37" s="92"/>
       <c r="M37" s="7"/>
     </row>
     <row r="38" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="M38" s="7"/>
     </row>
     <row r="39" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C39" s="120" t="s">
+      <c r="C39" s="93" t="s">
         <v>119</v>
       </c>
-      <c r="D39" s="121"/>
-      <c r="E39" s="121"/>
-      <c r="F39" s="122"/>
+      <c r="D39" s="94"/>
+      <c r="E39" s="94"/>
+      <c r="F39" s="95"/>
       <c r="G39" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="H39" s="120" t="s">
+      <c r="H39" s="93" t="s">
         <v>121</v>
       </c>
-      <c r="I39" s="123"/>
-      <c r="J39" s="121"/>
-      <c r="K39" s="121"/>
-      <c r="L39" s="122"/>
-      <c r="M39" s="120" t="s">
+      <c r="I39" s="96"/>
+      <c r="J39" s="94"/>
+      <c r="K39" s="94"/>
+      <c r="L39" s="95"/>
+      <c r="M39" s="93" t="s">
         <v>122</v>
       </c>
-      <c r="N39" s="123"/>
-      <c r="O39" s="121"/>
-      <c r="P39" s="122"/>
+      <c r="N39" s="96"/>
+      <c r="O39" s="94"/>
+      <c r="P39" s="95"/>
     </row>
     <row r="40" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="124" t="s">
+      <c r="B40" s="97" t="s">
         <v>105</v>
       </c>
-      <c r="C40" s="125" t="s">
+      <c r="C40" s="98" t="s">
         <v>123</v>
       </c>
-      <c r="D40" s="126" t="s">
+      <c r="D40" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="E40" s="126" t="s">
+      <c r="E40" s="90" t="s">
         <v>125</v>
       </c>
-      <c r="F40" s="127" t="s">
+      <c r="F40" s="91" t="s">
         <v>126</v>
       </c>
-      <c r="G40" s="128" t="s">
+      <c r="G40" s="99" t="s">
         <v>127</v>
       </c>
-      <c r="H40" s="137" t="s">
+      <c r="H40" s="86" t="s">
         <v>128</v>
       </c>
-      <c r="I40" s="138"/>
-      <c r="J40" s="126" t="s">
+      <c r="I40" s="87"/>
+      <c r="J40" s="90" t="s">
         <v>123</v>
       </c>
-      <c r="K40" s="126" t="s">
+      <c r="K40" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="L40" s="127" t="s">
+      <c r="L40" s="91" t="s">
         <v>125</v>
       </c>
-      <c r="M40" s="141" t="s">
+      <c r="M40" s="100" t="s">
         <v>128</v>
       </c>
-      <c r="N40" s="126" t="s">
+      <c r="N40" s="90" t="s">
         <v>123</v>
       </c>
-      <c r="O40" s="126" t="s">
+      <c r="O40" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="P40" s="127" t="s">
+      <c r="P40" s="91" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="41" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B41" s="124"/>
-      <c r="C41" s="125"/>
-      <c r="D41" s="126"/>
-      <c r="E41" s="126"/>
-      <c r="F41" s="127"/>
-      <c r="G41" s="128"/>
-      <c r="H41" s="139"/>
-      <c r="I41" s="140"/>
-      <c r="J41" s="126"/>
-      <c r="K41" s="126"/>
-      <c r="L41" s="127"/>
-      <c r="M41" s="142"/>
-      <c r="N41" s="126"/>
-      <c r="O41" s="126"/>
-      <c r="P41" s="127"/>
+      <c r="B41" s="97"/>
+      <c r="C41" s="98"/>
+      <c r="D41" s="90"/>
+      <c r="E41" s="90"/>
+      <c r="F41" s="91"/>
+      <c r="G41" s="99"/>
+      <c r="H41" s="88"/>
+      <c r="I41" s="89"/>
+      <c r="J41" s="90"/>
+      <c r="K41" s="90"/>
+      <c r="L41" s="91"/>
+      <c r="M41" s="101"/>
+      <c r="N41" s="90"/>
+      <c r="O41" s="90"/>
+      <c r="P41" s="91"/>
     </row>
     <row r="42" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B42" s="42" t="s">
@@ -5337,10 +5337,10 @@
       </c>
       <c r="F42" s="41"/>
       <c r="G42" s="46"/>
-      <c r="H42" s="133" t="s">
+      <c r="H42" s="80" t="s">
         <v>129</v>
       </c>
-      <c r="I42" s="134"/>
+      <c r="I42" s="81"/>
       <c r="J42" s="2">
         <v>3</v>
       </c>
@@ -5368,15 +5368,17 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="H40:I41"/>
-    <mergeCell ref="J40:J41"/>
-    <mergeCell ref="K40:K41"/>
-    <mergeCell ref="L40:L41"/>
-    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="C6:C35"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K11:L11"/>
     <mergeCell ref="C39:F39"/>
     <mergeCell ref="H39:L39"/>
     <mergeCell ref="M39:P39"/>
@@ -5390,17 +5392,15 @@
     <mergeCell ref="P40:P41"/>
     <mergeCell ref="M40:M41"/>
     <mergeCell ref="N40:N41"/>
-    <mergeCell ref="C6:C35"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="H40:I41"/>
+    <mergeCell ref="J40:J41"/>
+    <mergeCell ref="K40:K41"/>
+    <mergeCell ref="L40:L41"/>
+    <mergeCell ref="K37:L37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -5431,43 +5431,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="83"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="106"/>
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="88"/>
+      <c r="C3" s="130"/>
+      <c r="D3" s="130"/>
+      <c r="E3" s="130"/>
+      <c r="F3" s="130"/>
+      <c r="G3" s="131"/>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="89" t="s">
+      <c r="B5" s="132" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="89"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="89"/>
-      <c r="G5" s="90" t="s">
+      <c r="C5" s="132"/>
+      <c r="D5" s="132"/>
+      <c r="E5" s="132"/>
+      <c r="G5" s="133" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
-      <c r="K5" s="90"/>
-      <c r="L5" s="90"/>
-      <c r="M5" s="90"/>
-      <c r="N5" s="90"/>
-      <c r="O5" s="90"/>
-      <c r="P5" s="90"/>
-      <c r="Q5" s="90"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="133"/>
+      <c r="K5" s="133"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="133"/>
+      <c r="N5" s="133"/>
+      <c r="O5" s="133"/>
+      <c r="P5" s="133"/>
+      <c r="Q5" s="133"/>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6" s="23" t="s">
@@ -5482,20 +5482,20 @@
       <c r="E6" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="108" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="93" t="s">
+      <c r="H6" s="114" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="95" t="s">
+      <c r="I6" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="96"/>
-      <c r="K6" s="96"/>
-      <c r="L6" s="96"/>
-      <c r="M6" s="96"/>
-      <c r="N6" s="96"/>
+      <c r="J6" s="117"/>
+      <c r="K6" s="117"/>
+      <c r="L6" s="117"/>
+      <c r="M6" s="117"/>
+      <c r="N6" s="117"/>
       <c r="O6" s="118"/>
       <c r="P6" s="119" t="s">
         <v>30</v>
@@ -5506,15 +5506,15 @@
       <c r="B7" s="4">
         <v>1</v>
       </c>
-      <c r="C7" s="97" t="s">
+      <c r="C7" s="124" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>31</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="G7" s="92"/>
-      <c r="H7" s="94"/>
+      <c r="G7" s="134"/>
+      <c r="H7" s="135"/>
       <c r="I7" s="23" t="s">
         <v>32</v>
       </c>
@@ -5530,11 +5530,11 @@
       <c r="M7" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="N7" s="95" t="s">
+      <c r="N7" s="116" t="s">
         <v>37</v>
       </c>
       <c r="O7" s="118"/>
-      <c r="P7" s="95" t="s">
+      <c r="P7" s="116" t="s">
         <v>38</v>
       </c>
       <c r="Q7" s="118"/>
@@ -5543,7 +5543,7 @@
       <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="97"/>
+      <c r="C8" s="124"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
         <v>39</v>
@@ -5569,22 +5569,22 @@
       <c r="M8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="N8" s="144" t="s">
+      <c r="N8" s="152" t="s">
         <v>45</v>
       </c>
-      <c r="O8" s="145" t="s">
+      <c r="O8" s="153" t="s">
         <v>46</v>
       </c>
-      <c r="P8" s="144" t="s">
+      <c r="P8" s="152" t="s">
         <v>47</v>
       </c>
-      <c r="Q8" s="145"/>
+      <c r="Q8" s="153"/>
     </row>
     <row r="9" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="97" t="s">
+      <c r="C9" s="124" t="s">
         <v>48</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -5612,22 +5612,22 @@
       <c r="M9" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N9" s="144" t="s">
+      <c r="N9" s="152" t="s">
         <v>49</v>
       </c>
-      <c r="O9" s="145" t="s">
+      <c r="O9" s="153" t="s">
         <v>51</v>
       </c>
-      <c r="P9" s="144" t="s">
+      <c r="P9" s="152" t="s">
         <v>49</v>
       </c>
-      <c r="Q9" s="145"/>
+      <c r="Q9" s="153"/>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="97"/>
+      <c r="C10" s="124"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>52</v>
@@ -5653,20 +5653,20 @@
       <c r="M10" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="N10" s="150" t="s">
+      <c r="N10" s="146" t="s">
         <v>45</v>
       </c>
-      <c r="O10" s="151"/>
-      <c r="P10" s="150" t="s">
+      <c r="O10" s="147"/>
+      <c r="P10" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="Q10" s="151"/>
+      <c r="Q10" s="147"/>
     </row>
     <row r="11" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="97" t="s">
+      <c r="C11" s="124" t="s">
         <v>56</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -5694,20 +5694,20 @@
       <c r="M11" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="N11" s="150" t="s">
+      <c r="N11" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="O11" s="151"/>
-      <c r="P11" s="150" t="s">
+      <c r="O11" s="147"/>
+      <c r="P11" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="Q11" s="151"/>
+      <c r="Q11" s="147"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="97"/>
+      <c r="C12" s="124"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
         <v>58</v>
@@ -5746,7 +5746,7 @@
       <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="99" t="s">
+      <c r="C13" s="126" t="s">
         <v>62</v>
       </c>
       <c r="D13" s="4" t="s">
@@ -5787,7 +5787,7 @@
       <c r="B14" s="4">
         <v>8</v>
       </c>
-      <c r="C14" s="100"/>
+      <c r="C14" s="127"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
         <v>63</v>
@@ -5813,18 +5813,18 @@
       <c r="M14" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="N14" s="152" t="s">
+      <c r="N14" s="144" t="s">
         <v>64</v>
       </c>
-      <c r="O14" s="153"/>
-      <c r="P14" s="146"/>
-      <c r="Q14" s="147"/>
+      <c r="O14" s="145"/>
+      <c r="P14" s="150"/>
+      <c r="Q14" s="151"/>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B15" s="4">
         <v>9</v>
       </c>
-      <c r="C15" s="97" t="s">
+      <c r="C15" s="124" t="s">
         <v>49</v>
       </c>
       <c r="D15" s="4"/>
@@ -5840,16 +5840,16 @@
       <c r="K15" s="18"/>
       <c r="L15" s="18"/>
       <c r="M15" s="18"/>
-      <c r="N15" s="144"/>
-      <c r="O15" s="145"/>
-      <c r="P15" s="146"/>
-      <c r="Q15" s="147"/>
+      <c r="N15" s="152"/>
+      <c r="O15" s="153"/>
+      <c r="P15" s="150"/>
+      <c r="Q15" s="151"/>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" s="4">
         <v>10</v>
       </c>
-      <c r="C16" s="97"/>
+      <c r="C16" s="124"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="G16" s="19"/>
@@ -5859,16 +5859,16 @@
       <c r="K16" s="18"/>
       <c r="L16" s="18"/>
       <c r="M16" s="18"/>
-      <c r="N16" s="144"/>
-      <c r="O16" s="145"/>
-      <c r="P16" s="146"/>
-      <c r="Q16" s="147"/>
+      <c r="N16" s="152"/>
+      <c r="O16" s="153"/>
+      <c r="P16" s="150"/>
+      <c r="Q16" s="151"/>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="4">
         <v>11</v>
       </c>
-      <c r="C17" s="97" t="s">
+      <c r="C17" s="124" t="s">
         <v>49</v>
       </c>
       <c r="D17" s="4"/>
@@ -5880,16 +5880,16 @@
       <c r="K17" s="18"/>
       <c r="L17" s="18"/>
       <c r="M17" s="18"/>
-      <c r="N17" s="144"/>
-      <c r="O17" s="145"/>
-      <c r="P17" s="146"/>
-      <c r="Q17" s="147"/>
+      <c r="N17" s="152"/>
+      <c r="O17" s="153"/>
+      <c r="P17" s="150"/>
+      <c r="Q17" s="151"/>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="4">
         <v>12</v>
       </c>
-      <c r="C18" s="97"/>
+      <c r="C18" s="124"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="G18" s="19"/>
@@ -5899,16 +5899,16 @@
       <c r="K18" s="18"/>
       <c r="L18" s="18"/>
       <c r="M18" s="18"/>
-      <c r="N18" s="144"/>
-      <c r="O18" s="145"/>
-      <c r="P18" s="146"/>
-      <c r="Q18" s="147"/>
+      <c r="N18" s="152"/>
+      <c r="O18" s="153"/>
+      <c r="P18" s="150"/>
+      <c r="Q18" s="151"/>
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="4">
         <v>13</v>
       </c>
-      <c r="C19" s="97" t="s">
+      <c r="C19" s="124" t="s">
         <v>49</v>
       </c>
       <c r="D19" s="4"/>
@@ -5920,16 +5920,16 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
-      <c r="N19" s="144"/>
-      <c r="O19" s="145"/>
-      <c r="P19" s="146"/>
-      <c r="Q19" s="147"/>
+      <c r="N19" s="152"/>
+      <c r="O19" s="153"/>
+      <c r="P19" s="150"/>
+      <c r="Q19" s="151"/>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="4">
         <v>14</v>
       </c>
-      <c r="C20" s="97"/>
+      <c r="C20" s="124"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
@@ -5937,11 +5937,36 @@
       <c r="D22" t="s">
         <v>65</v>
       </c>
-      <c r="F22" s="98"/>
-      <c r="G22" s="98"/>
+      <c r="F22" s="125"/>
+      <c r="G22" s="125"/>
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="P19:Q19"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="I6:O6"/>
+    <mergeCell ref="N8:O8"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C7:C8"/>
@@ -5958,31 +5983,6 @@
     <mergeCell ref="P10:Q10"/>
     <mergeCell ref="P11:Q11"/>
     <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="N7:O7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="I6:O6"/>
-    <mergeCell ref="N8:O8"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="P15:Q15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6015,44 +6015,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="83"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="106"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="88"/>
+      <c r="C3" s="130"/>
+      <c r="D3" s="130"/>
+      <c r="E3" s="130"/>
+      <c r="F3" s="130"/>
+      <c r="G3" s="131"/>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B5" s="106" t="s">
+      <c r="B5" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="106"/>
-      <c r="D5" s="106"/>
+      <c r="C5" s="141"/>
+      <c r="D5" s="141"/>
       <c r="E5" s="3"/>
-      <c r="G5" s="90" t="s">
+      <c r="G5" s="133" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="90"/>
-      <c r="I5" s="90"/>
-      <c r="J5" s="90"/>
-      <c r="K5" s="90"/>
-      <c r="L5" s="90"/>
-      <c r="M5" s="90"/>
-      <c r="N5" s="90"/>
-      <c r="O5" s="90"/>
-      <c r="P5" s="90"/>
-      <c r="Q5" s="90"/>
-      <c r="R5" s="90"/>
+      <c r="H5" s="133"/>
+      <c r="I5" s="133"/>
+      <c r="J5" s="133"/>
+      <c r="K5" s="133"/>
+      <c r="L5" s="133"/>
+      <c r="M5" s="133"/>
+      <c r="N5" s="133"/>
+      <c r="O5" s="133"/>
+      <c r="P5" s="133"/>
+      <c r="Q5" s="133"/>
+      <c r="R5" s="133"/>
     </row>
     <row r="6" spans="2:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
@@ -6065,45 +6065,45 @@
         <v>66</v>
       </c>
       <c r="E6" s="10"/>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="108" t="s">
         <v>69</v>
       </c>
-      <c r="H6" s="91" t="s">
+      <c r="H6" s="108" t="s">
         <v>70</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="108" t="s">
         <v>71</v>
       </c>
-      <c r="J6" s="93" t="s">
+      <c r="J6" s="114" t="s">
         <v>72</v>
       </c>
-      <c r="K6" s="107" t="s">
+      <c r="K6" s="142" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="108"/>
-      <c r="M6" s="108"/>
-      <c r="N6" s="108"/>
-      <c r="O6" s="108"/>
+      <c r="L6" s="143"/>
+      <c r="M6" s="143"/>
+      <c r="N6" s="143"/>
+      <c r="O6" s="143"/>
       <c r="P6" s="156"/>
-      <c r="Q6" s="107" t="s">
+      <c r="Q6" s="142" t="s">
         <v>30</v>
       </c>
       <c r="R6" s="156"/>
     </row>
     <row r="7" spans="2:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="B7" s="99">
+      <c r="B7" s="126">
         <v>1</v>
       </c>
-      <c r="C7" s="102" t="s">
+      <c r="C7" s="137" t="s">
         <v>73</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G7" s="92"/>
-      <c r="H7" s="92"/>
-      <c r="I7" s="92"/>
-      <c r="J7" s="94"/>
+      <c r="G7" s="134"/>
+      <c r="H7" s="134"/>
+      <c r="I7" s="134"/>
+      <c r="J7" s="135"/>
       <c r="K7" s="23" t="s">
         <v>32</v>
       </c>
@@ -6122,14 +6122,14 @@
       <c r="P7" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="Q7" s="95" t="s">
+      <c r="Q7" s="116" t="s">
         <v>75</v>
       </c>
       <c r="R7" s="118"/>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B8" s="101"/>
-      <c r="C8" s="103"/>
+      <c r="B8" s="136"/>
+      <c r="C8" s="138"/>
       <c r="D8" s="2" t="s">
         <v>76</v>
       </c>
@@ -6149,12 +6149,12 @@
       <c r="N8" s="34"/>
       <c r="O8" s="34"/>
       <c r="P8" s="34"/>
-      <c r="Q8" s="154"/>
-      <c r="R8" s="155"/>
+      <c r="Q8" s="157"/>
+      <c r="R8" s="158"/>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="101"/>
-      <c r="C9" s="103"/>
+      <c r="B9" s="136"/>
+      <c r="C9" s="138"/>
       <c r="D9" s="2" t="s">
         <v>78</v>
       </c>
@@ -6190,8 +6190,8 @@
       <c r="R9" s="149"/>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="101"/>
-      <c r="C10" s="103"/>
+      <c r="B10" s="136"/>
+      <c r="C10" s="138"/>
       <c r="D10" s="2" t="s">
         <v>80</v>
       </c>
@@ -6221,14 +6221,14 @@
       <c r="P10" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="Q10" s="154" t="s">
+      <c r="Q10" s="157" t="s">
         <v>47</v>
       </c>
-      <c r="R10" s="155"/>
+      <c r="R10" s="158"/>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B11" s="101"/>
-      <c r="C11" s="103"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="138"/>
       <c r="D11" s="2" t="s">
         <v>84</v>
       </c>
@@ -6258,14 +6258,14 @@
       <c r="P11" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="Q11" s="154" t="s">
+      <c r="Q11" s="157" t="s">
         <v>47</v>
       </c>
-      <c r="R11" s="155"/>
+      <c r="R11" s="158"/>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B12" s="100"/>
-      <c r="C12" s="104"/>
+      <c r="B12" s="127"/>
+      <c r="C12" s="139"/>
       <c r="D12" s="2" t="s">
         <v>86</v>
       </c>
@@ -6295,16 +6295,16 @@
       <c r="P12" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="Q12" s="154" t="s">
+      <c r="Q12" s="157" t="s">
         <v>47</v>
       </c>
-      <c r="R12" s="155"/>
+      <c r="R12" s="158"/>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B13" s="99">
+      <c r="B13" s="126">
         <v>2</v>
       </c>
-      <c r="C13" s="99" t="s">
+      <c r="C13" s="126" t="s">
         <v>88</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -6344,8 +6344,8 @@
       <c r="R13" s="149"/>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B14" s="101"/>
-      <c r="C14" s="101"/>
+      <c r="B14" s="136"/>
+      <c r="C14" s="136"/>
       <c r="D14" s="2" t="s">
         <v>91</v>
       </c>
@@ -6367,12 +6367,12 @@
       <c r="N14" s="34"/>
       <c r="O14" s="34"/>
       <c r="P14" s="34"/>
-      <c r="Q14" s="154"/>
-      <c r="R14" s="155"/>
+      <c r="Q14" s="157"/>
+      <c r="R14" s="158"/>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B15" s="101"/>
-      <c r="C15" s="101"/>
+      <c r="B15" s="136"/>
+      <c r="C15" s="136"/>
       <c r="D15" s="2" t="s">
         <v>92</v>
       </c>
@@ -6394,12 +6394,12 @@
       <c r="N15" s="34"/>
       <c r="O15" s="34"/>
       <c r="P15" s="34"/>
-      <c r="Q15" s="154"/>
-      <c r="R15" s="155"/>
+      <c r="Q15" s="157"/>
+      <c r="R15" s="158"/>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B16" s="101"/>
-      <c r="C16" s="101"/>
+      <c r="B16" s="136"/>
+      <c r="C16" s="136"/>
       <c r="D16" s="2" t="s">
         <v>93</v>
       </c>
@@ -6415,12 +6415,12 @@
       <c r="N16" s="34"/>
       <c r="O16" s="34"/>
       <c r="P16" s="34"/>
-      <c r="Q16" s="154"/>
-      <c r="R16" s="155"/>
+      <c r="Q16" s="157"/>
+      <c r="R16" s="158"/>
     </row>
     <row r="17" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B17" s="101"/>
-      <c r="C17" s="101"/>
+      <c r="B17" s="136"/>
+      <c r="C17" s="136"/>
       <c r="D17" s="2" t="s">
         <v>94</v>
       </c>
@@ -6436,12 +6436,12 @@
       <c r="N17" s="34"/>
       <c r="O17" s="34"/>
       <c r="P17" s="34"/>
-      <c r="Q17" s="154"/>
-      <c r="R17" s="155"/>
+      <c r="Q17" s="157"/>
+      <c r="R17" s="158"/>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B18" s="100"/>
-      <c r="C18" s="100"/>
+      <c r="B18" s="127"/>
+      <c r="C18" s="127"/>
       <c r="D18" s="2" t="s">
         <v>95</v>
       </c>
@@ -6457,14 +6457,14 @@
       <c r="N18" s="34"/>
       <c r="O18" s="34"/>
       <c r="P18" s="34"/>
-      <c r="Q18" s="154"/>
-      <c r="R18" s="155"/>
+      <c r="Q18" s="157"/>
+      <c r="R18" s="158"/>
     </row>
     <row r="19" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B19" s="99">
+      <c r="B19" s="126">
         <v>3</v>
       </c>
-      <c r="C19" s="102" t="s">
+      <c r="C19" s="137" t="s">
         <v>96</v>
       </c>
       <c r="D19" s="2" t="s">
@@ -6482,12 +6482,12 @@
       <c r="N19" s="34"/>
       <c r="O19" s="34"/>
       <c r="P19" s="34"/>
-      <c r="Q19" s="154"/>
-      <c r="R19" s="155"/>
+      <c r="Q19" s="157"/>
+      <c r="R19" s="158"/>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B20" s="101"/>
-      <c r="C20" s="103"/>
+      <c r="B20" s="136"/>
+      <c r="C20" s="138"/>
       <c r="D20" s="2" t="s">
         <v>98</v>
       </c>
@@ -6503,12 +6503,12 @@
       <c r="N20" s="34"/>
       <c r="O20" s="34"/>
       <c r="P20" s="34"/>
-      <c r="Q20" s="154"/>
-      <c r="R20" s="155"/>
+      <c r="Q20" s="157"/>
+      <c r="R20" s="158"/>
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B21" s="101"/>
-      <c r="C21" s="103"/>
+      <c r="B21" s="136"/>
+      <c r="C21" s="138"/>
       <c r="D21" s="2" t="s">
         <v>99</v>
       </c>
@@ -6524,12 +6524,12 @@
       <c r="N21" s="34"/>
       <c r="O21" s="34"/>
       <c r="P21" s="34"/>
-      <c r="Q21" s="154"/>
-      <c r="R21" s="155"/>
+      <c r="Q21" s="157"/>
+      <c r="R21" s="158"/>
     </row>
     <row r="22" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B22" s="101"/>
-      <c r="C22" s="103"/>
+      <c r="B22" s="136"/>
+      <c r="C22" s="138"/>
       <c r="D22" s="2" t="s">
         <v>100</v>
       </c>
@@ -6545,12 +6545,12 @@
       <c r="N22" s="34"/>
       <c r="O22" s="34"/>
       <c r="P22" s="34"/>
-      <c r="Q22" s="154"/>
-      <c r="R22" s="155"/>
+      <c r="Q22" s="157"/>
+      <c r="R22" s="158"/>
     </row>
     <row r="23" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B23" s="101"/>
-      <c r="C23" s="103"/>
+      <c r="B23" s="136"/>
+      <c r="C23" s="138"/>
       <c r="D23" s="2" t="s">
         <v>101</v>
       </c>
@@ -6566,12 +6566,12 @@
       <c r="N23" s="34"/>
       <c r="O23" s="34"/>
       <c r="P23" s="34"/>
-      <c r="Q23" s="154"/>
-      <c r="R23" s="155"/>
+      <c r="Q23" s="157"/>
+      <c r="R23" s="158"/>
     </row>
     <row r="24" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B24" s="100"/>
-      <c r="C24" s="104"/>
+      <c r="B24" s="127"/>
+      <c r="C24" s="139"/>
       <c r="D24" s="2" t="s">
         <v>102</v>
       </c>
@@ -6587,14 +6587,14 @@
       <c r="N24" s="34"/>
       <c r="O24" s="34"/>
       <c r="P24" s="34"/>
-      <c r="Q24" s="154"/>
-      <c r="R24" s="155"/>
+      <c r="Q24" s="157"/>
+      <c r="R24" s="158"/>
     </row>
     <row r="25" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B25" s="99">
+      <c r="B25" s="126">
         <v>4</v>
       </c>
-      <c r="C25" s="102" t="s">
+      <c r="C25" s="137" t="s">
         <v>49</v>
       </c>
       <c r="D25" s="2" t="s">
@@ -6612,60 +6612,84 @@
       <c r="N25" s="34"/>
       <c r="O25" s="34"/>
       <c r="P25" s="34"/>
-      <c r="Q25" s="154"/>
-      <c r="R25" s="155"/>
+      <c r="Q25" s="157"/>
+      <c r="R25" s="158"/>
     </row>
     <row r="26" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B26" s="101"/>
-      <c r="C26" s="103"/>
+      <c r="B26" s="136"/>
+      <c r="C26" s="138"/>
       <c r="D26" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="27" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B27" s="101"/>
-      <c r="C27" s="103"/>
+      <c r="B27" s="136"/>
+      <c r="C27" s="138"/>
       <c r="D27" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="28" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B28" s="101"/>
-      <c r="C28" s="103"/>
+      <c r="B28" s="136"/>
+      <c r="C28" s="138"/>
       <c r="D28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G28" s="98"/>
-      <c r="H28" s="98"/>
-      <c r="I28" s="157"/>
-      <c r="J28" s="157"/>
-      <c r="K28" s="157"/>
-      <c r="L28" s="157"/>
-      <c r="M28" s="157"/>
+      <c r="G28" s="125"/>
+      <c r="H28" s="125"/>
+      <c r="I28" s="155"/>
+      <c r="J28" s="155"/>
+      <c r="K28" s="155"/>
+      <c r="L28" s="155"/>
+      <c r="M28" s="155"/>
       <c r="N28" s="43"/>
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B29" s="101"/>
-      <c r="C29" s="103"/>
+      <c r="B29" s="136"/>
+      <c r="C29" s="138"/>
       <c r="D29" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="I29" s="158"/>
-      <c r="J29" s="158"/>
-      <c r="K29" s="158"/>
-      <c r="L29" s="158"/>
-      <c r="M29" s="158"/>
+      <c r="I29" s="154"/>
+      <c r="J29" s="154"/>
+      <c r="K29" s="154"/>
+      <c r="L29" s="154"/>
+      <c r="M29" s="154"/>
       <c r="N29" s="44"/>
     </row>
     <row r="30" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B30" s="100"/>
-      <c r="C30" s="104"/>
+      <c r="B30" s="127"/>
+      <c r="C30" s="139"/>
       <c r="D30" s="2" t="s">
         <v>49</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="K6:P6"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="I28:M28"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q9:R9"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="I6:I7"/>
@@ -6682,30 +6706,6 @@
     <mergeCell ref="G5:R5"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="I28:M28"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="K6:P6"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="Q12:R12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6732,51 +6732,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="104" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="83"/>
+      <c r="C1" s="105"/>
+      <c r="D1" s="105"/>
+      <c r="E1" s="106"/>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B3" s="111" t="s">
+      <c r="B3" s="107" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
-      <c r="M3" s="111"/>
-      <c r="N3" s="111"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="107"/>
+      <c r="L3" s="107"/>
+      <c r="M3" s="107"/>
+      <c r="N3" s="107"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="108" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="113" t="s">
+      <c r="C4" s="110" t="s">
         <v>105</v>
       </c>
-      <c r="D4" s="115" t="s">
+      <c r="D4" s="112" t="s">
         <v>106</v>
       </c>
-      <c r="E4" s="93" t="s">
+      <c r="E4" s="114" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="95" t="s">
+      <c r="F4" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="96"/>
-      <c r="H4" s="96"/>
-      <c r="I4" s="96"/>
-      <c r="J4" s="96"/>
-      <c r="K4" s="96"/>
+      <c r="G4" s="117"/>
+      <c r="H4" s="117"/>
+      <c r="I4" s="117"/>
+      <c r="J4" s="117"/>
+      <c r="K4" s="117"/>
       <c r="L4" s="118"/>
       <c r="M4" s="119" t="s">
         <v>30</v>
@@ -6784,10 +6784,10 @@
       <c r="N4" s="119"/>
     </row>
     <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="112"/>
-      <c r="C5" s="114"/>
-      <c r="D5" s="116"/>
-      <c r="E5" s="117"/>
+      <c r="B5" s="109"/>
+      <c r="C5" s="111"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="115"/>
       <c r="F5" s="26" t="s">
         <v>32</v>
       </c>
@@ -6818,7 +6818,7 @@
       <c r="B6" s="24">
         <v>1</v>
       </c>
-      <c r="C6" s="109" t="s">
+      <c r="C6" s="102" t="s">
         <v>109</v>
       </c>
       <c r="D6" s="30" t="s">
@@ -6860,7 +6860,7 @@
         <f>B6+1</f>
         <v>2</v>
       </c>
-      <c r="C7" s="109"/>
+      <c r="C7" s="102"/>
       <c r="D7" s="31" t="s">
         <v>112</v>
       </c>
@@ -6898,7 +6898,7 @@
         <f t="shared" ref="B8:B13" si="0">B7+1</f>
         <v>3</v>
       </c>
-      <c r="C8" s="109"/>
+      <c r="C8" s="102"/>
       <c r="D8" s="31" t="s">
         <v>114</v>
       </c>
@@ -6936,7 +6936,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C9" s="109"/>
+      <c r="C9" s="102"/>
       <c r="D9" s="31" t="s">
         <v>49</v>
       </c>
@@ -6958,10 +6958,10 @@
       <c r="J9" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K9" s="131" t="s">
+      <c r="K9" s="120" t="s">
         <v>49</v>
       </c>
-      <c r="L9" s="132"/>
+      <c r="L9" s="121"/>
       <c r="M9" s="12" t="s">
         <v>49</v>
       </c>
@@ -6974,7 +6974,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C10" s="109"/>
+      <c r="C10" s="102"/>
       <c r="D10" s="31" t="s">
         <v>51</v>
       </c>
@@ -6996,10 +6996,10 @@
       <c r="J10" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="K10" s="129" t="s">
+      <c r="K10" s="84" t="s">
         <v>45</v>
       </c>
-      <c r="L10" s="130"/>
+      <c r="L10" s="85"/>
       <c r="M10" s="6" t="s">
         <v>61</v>
       </c>
@@ -7012,7 +7012,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C11" s="109"/>
+      <c r="C11" s="102"/>
       <c r="D11" s="31" t="s">
         <v>51</v>
       </c>
@@ -7034,10 +7034,10 @@
       <c r="J11" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="K11" s="129" t="s">
+      <c r="K11" s="84" t="s">
         <v>45</v>
       </c>
-      <c r="L11" s="130"/>
+      <c r="L11" s="85"/>
       <c r="M11" s="5" t="s">
         <v>47</v>
       </c>
@@ -7050,7 +7050,7 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C12" s="109"/>
+      <c r="C12" s="102"/>
       <c r="D12" s="31" t="s">
         <v>51</v>
       </c>
@@ -7072,10 +7072,10 @@
       <c r="J12" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="K12" s="129" t="s">
+      <c r="K12" s="84" t="s">
         <v>45</v>
       </c>
-      <c r="L12" s="130"/>
+      <c r="L12" s="85"/>
       <c r="M12" s="5" t="s">
         <v>47</v>
       </c>
@@ -7088,7 +7088,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C13" s="110"/>
+      <c r="C13" s="103"/>
       <c r="D13" s="32" t="s">
         <v>49</v>
       </c>
@@ -7110,10 +7110,10 @@
       <c r="J13" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="K13" s="135" t="s">
+      <c r="K13" s="82" t="s">
         <v>49</v>
       </c>
-      <c r="L13" s="136"/>
+      <c r="L13" s="83"/>
       <c r="M13" s="25" t="s">
         <v>49</v>
       </c>
@@ -7148,98 +7148,98 @@
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
-      <c r="K15" s="143"/>
-      <c r="L15" s="143"/>
+      <c r="K15" s="92"/>
+      <c r="L15" s="92"/>
       <c r="M15" s="7"/>
     </row>
     <row r="16" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="M16" s="7"/>
     </row>
     <row r="17" spans="2:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="120" t="s">
+      <c r="C17" s="93" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="121"/>
-      <c r="E17" s="121"/>
-      <c r="F17" s="122"/>
+      <c r="D17" s="94"/>
+      <c r="E17" s="94"/>
+      <c r="F17" s="95"/>
       <c r="G17" s="39" t="s">
         <v>120</v>
       </c>
-      <c r="H17" s="120" t="s">
+      <c r="H17" s="93" t="s">
         <v>121</v>
       </c>
-      <c r="I17" s="123"/>
-      <c r="J17" s="121"/>
-      <c r="K17" s="121"/>
-      <c r="L17" s="122"/>
-      <c r="M17" s="120" t="s">
+      <c r="I17" s="96"/>
+      <c r="J17" s="94"/>
+      <c r="K17" s="94"/>
+      <c r="L17" s="95"/>
+      <c r="M17" s="93" t="s">
         <v>122</v>
       </c>
-      <c r="N17" s="123"/>
-      <c r="O17" s="121"/>
-      <c r="P17" s="122"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="94"/>
+      <c r="P17" s="95"/>
     </row>
     <row r="18" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="124" t="s">
+      <c r="B18" s="97" t="s">
         <v>105</v>
       </c>
-      <c r="C18" s="125" t="s">
+      <c r="C18" s="98" t="s">
         <v>123</v>
       </c>
-      <c r="D18" s="126" t="s">
+      <c r="D18" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="E18" s="126" t="s">
+      <c r="E18" s="90" t="s">
         <v>125</v>
       </c>
-      <c r="F18" s="127" t="s">
+      <c r="F18" s="91" t="s">
         <v>126</v>
       </c>
-      <c r="G18" s="128" t="s">
+      <c r="G18" s="99" t="s">
         <v>127</v>
       </c>
-      <c r="H18" s="137" t="s">
+      <c r="H18" s="86" t="s">
         <v>128</v>
       </c>
-      <c r="I18" s="138"/>
-      <c r="J18" s="126" t="s">
+      <c r="I18" s="87"/>
+      <c r="J18" s="90" t="s">
         <v>123</v>
       </c>
-      <c r="K18" s="126" t="s">
+      <c r="K18" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="L18" s="127" t="s">
+      <c r="L18" s="91" t="s">
         <v>125</v>
       </c>
-      <c r="M18" s="141" t="s">
+      <c r="M18" s="100" t="s">
         <v>128</v>
       </c>
-      <c r="N18" s="126" t="s">
+      <c r="N18" s="90" t="s">
         <v>123</v>
       </c>
-      <c r="O18" s="126" t="s">
+      <c r="O18" s="90" t="s">
         <v>124</v>
       </c>
-      <c r="P18" s="127" t="s">
+      <c r="P18" s="91" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B19" s="124"/>
-      <c r="C19" s="125"/>
-      <c r="D19" s="126"/>
-      <c r="E19" s="126"/>
-      <c r="F19" s="127"/>
-      <c r="G19" s="128"/>
-      <c r="H19" s="139"/>
-      <c r="I19" s="140"/>
-      <c r="J19" s="126"/>
-      <c r="K19" s="126"/>
-      <c r="L19" s="127"/>
-      <c r="M19" s="142"/>
-      <c r="N19" s="126"/>
-      <c r="O19" s="126"/>
-      <c r="P19" s="127"/>
+      <c r="B19" s="97"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="90"/>
+      <c r="E19" s="90"/>
+      <c r="F19" s="91"/>
+      <c r="G19" s="99"/>
+      <c r="H19" s="88"/>
+      <c r="I19" s="89"/>
+      <c r="J19" s="90"/>
+      <c r="K19" s="90"/>
+      <c r="L19" s="91"/>
+      <c r="M19" s="101"/>
+      <c r="N19" s="90"/>
+      <c r="O19" s="90"/>
+      <c r="P19" s="91"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="42" t="s">
@@ -7256,10 +7256,10 @@
       </c>
       <c r="F20" s="41"/>
       <c r="G20" s="46"/>
-      <c r="H20" s="133" t="s">
+      <c r="H20" s="80" t="s">
         <v>129</v>
       </c>
-      <c r="I20" s="134"/>
+      <c r="I20" s="81"/>
       <c r="J20" s="2">
         <v>3</v>
       </c>
@@ -7287,20 +7287,12 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="L18:L19"/>
+    <mergeCell ref="O18:O19"/>
+    <mergeCell ref="P18:P19"/>
+    <mergeCell ref="M17:P17"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="N18:N19"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="C6:C13"/>
     <mergeCell ref="B4:B5"/>
@@ -7317,12 +7309,20 @@
     <mergeCell ref="H18:I19"/>
     <mergeCell ref="G18:G19"/>
     <mergeCell ref="K18:K19"/>
-    <mergeCell ref="L18:L19"/>
-    <mergeCell ref="O18:O19"/>
-    <mergeCell ref="P18:P19"/>
-    <mergeCell ref="M17:P17"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="N18:N19"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="B3:N3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7340,12 +7340,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E819BB071F23F542A5DF0E9C9037AD04" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="798a38e6de461387c626d04793181ea9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="301f98df-4edd-4096-94f8-2f8af3eee570" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b4b8dab68acb31e3ac71f6347d499c29" ns2:_="">
     <xsd:import namespace="301f98df-4edd-4096-94f8-2f8af3eee570"/>
@@ -7483,6 +7477,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83B9CA12-8961-4BEB-8D70-94D8CF82FF06}">
   <ds:schemaRefs>
@@ -7492,15 +7492,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47FE877D-432C-44A9-9889-489A1D266CB2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3E854E7-906F-4C7C-AFC0-1BC802AE88F0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7516,4 +7507,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47FE877D-432C-44A9-9889-489A1D266CB2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>